<commit_message>
Add all project code
</commit_message>
<xml_diff>
--- a/resources/templates/Checklist.xlsx
+++ b/resources/templates/Checklist.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="117">
   <si>
     <t>Checklist For Action in the Regional/Field Office</t>
   </si>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">SG/Step: </t>
   </si>
   <si>
-    <t>13-1</t>
+    <t>${salary_grade}</t>
   </si>
   <si>
     <t>Monthly Compensation</t>
@@ -237,7 +237,7 @@
     <t xml:space="preserve">         i. Provisional Appointment notation for DepEd </t>
   </si>
   <si>
-    <t>Permanent</t>
+    <t>${employment_status}</t>
   </si>
   <si>
     <t xml:space="preserve">        ii. Is the appointee subject for Probation?
@@ -248,13 +248,10 @@
     <t>Nature of Appointment</t>
   </si>
   <si>
-    <t>Promotion</t>
-  </si>
-  <si>
     <t>Signature of Appointing Authority</t>
   </si>
   <si>
-    <t>August 18, 2025</t>
+    <t>${date_signed}</t>
   </si>
   <si>
     <t>Date of Signing</t>
@@ -1227,18 +1224,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="8.5"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="8.5"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="8.5"/>
@@ -1285,13 +1280,6 @@
       <color theme="1"/>
       <name val="Bell MT"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1450,6 +1438,14 @@
       <i/>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8.5"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2428,146 +2424,146 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="30" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="55" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="4" borderId="55" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="56" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="57" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="5" borderId="58" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="5" borderId="58" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="6" borderId="59" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="6" borderId="59" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="6" borderId="58" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="6" borderId="58" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="41" fillId="7" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="7" borderId="60" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="61" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="61" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="62" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="62" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="46" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="47" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="48" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="47" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2836,10 +2832,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2866,14 +2862,14 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="176" fontId="24" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="24" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="23" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="23" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2912,7 +2908,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2930,7 +2926,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2991,7 +2987,7 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3054,7 +3050,7 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="1" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3069,7 +3065,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3084,7 +3080,7 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3105,10 +3101,10 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3240,9 +3236,6 @@
     <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3264,10 +3257,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="24" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
@@ -3276,13 +3266,13 @@
     <xf numFmtId="176" fontId="1" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3355,7 +3345,7 @@
       <xdr:row>77</xdr:row>
       <xdr:rowOff>15249</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="168166" cy="151711"/>
+    <xdr:ext cx="168166" cy="159331"/>
     <xdr:sp>
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1"/>
@@ -3363,8 +3353,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="311150" y="21461730"/>
-          <a:ext cx="168275" cy="151130"/>
+          <a:off x="311150" y="21042630"/>
+          <a:ext cx="168275" cy="158750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3424,7 +3414,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="309880" y="21262975"/>
+          <a:off x="309880" y="20843875"/>
           <a:ext cx="168275" cy="165100"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3485,7 +3475,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="309245" y="21114385"/>
+          <a:off x="309245" y="20695285"/>
           <a:ext cx="168275" cy="167005"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3813,14 +3803,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:J87"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="13.4259259259259" style="4" customWidth="1"/>
+    <col min="1" max="1" width="13.425" style="4" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="57.712962962963" style="1" customWidth="1"/>
-    <col min="4" max="4" width="5.57407407407407" customWidth="1"/>
-    <col min="5" max="5" width="5.71296296296296" customWidth="1"/>
-    <col min="6" max="6" width="4.13888888888889" customWidth="1"/>
+    <col min="3" max="3" width="57.7166666666667" style="1" customWidth="1"/>
+    <col min="4" max="4" width="5.575" customWidth="1"/>
+    <col min="5" max="5" width="5.71666666666667" customWidth="1"/>
+    <col min="6" max="6" width="4.14166666666667" customWidth="1"/>
     <col min="7" max="9" width="4" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3890,7 +3880,7 @@
         <v>7</v>
       </c>
       <c r="E5" s="20"/>
-      <c r="F5" s="244" t="s">
+      <c r="F5" s="21" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="21"/>
@@ -3992,7 +3982,7 @@
       <c r="C11" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="245" t="s">
+      <c r="D11" s="244" t="s">
         <v>26</v>
       </c>
       <c r="E11" s="54"/>
@@ -4013,11 +4003,11 @@
       <c r="C12" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="246" t="s">
+      <c r="D12" s="245" t="s">
         <v>26</v>
       </c>
       <c r="E12" s="62"/>
-      <c r="F12" s="247" t="s">
+      <c r="F12" s="246" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="63"/>
@@ -4032,11 +4022,11 @@
       <c r="C13" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="246" t="s">
+      <c r="D13" s="245" t="s">
         <v>26</v>
       </c>
       <c r="E13" s="62"/>
-      <c r="F13" s="247" t="s">
+      <c r="F13" s="246" t="s">
         <v>30</v>
       </c>
       <c r="G13" s="63"/>
@@ -4051,11 +4041,11 @@
       <c r="C14" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="246" t="s">
+      <c r="D14" s="245" t="s">
         <v>26</v>
       </c>
       <c r="E14" s="61"/>
-      <c r="F14" s="248" t="s">
+      <c r="F14" s="247" t="s">
         <v>33</v>
       </c>
       <c r="G14" s="65"/>
@@ -4095,7 +4085,7 @@
       <c r="I16" s="75"/>
     </row>
     <row r="17" s="2" customFormat="1" ht="13.5" customHeight="1" spans="1:9">
-      <c r="A17" s="249" t="s">
+      <c r="A17" s="248" t="s">
         <v>37</v>
       </c>
       <c r="B17" s="77">
@@ -4132,7 +4122,7 @@
       <c r="C19" s="87" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="250" t="s">
+      <c r="D19" s="249" t="s">
         <v>26</v>
       </c>
       <c r="E19" s="79"/>
@@ -4253,7 +4243,7 @@
         <v>48</v>
       </c>
       <c r="D27" s="95"/>
-      <c r="E27" s="251" t="s">
+      <c r="E27" s="250" t="s">
         <v>26</v>
       </c>
       <c r="F27" s="96" t="s">
@@ -4270,7 +4260,7 @@
         <v>50</v>
       </c>
       <c r="D28" s="100"/>
-      <c r="E28" s="250" t="s">
+      <c r="E28" s="249" t="s">
         <v>26</v>
       </c>
       <c r="F28" s="101" t="s">
@@ -4288,12 +4278,12 @@
       <c r="C29" s="105" t="s">
         <v>51</v>
       </c>
-      <c r="D29" s="252" t="s">
+      <c r="D29" s="251" t="s">
         <v>26</v>
       </c>
       <c r="E29" s="107"/>
       <c r="F29" s="108" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="G29" s="108"/>
       <c r="H29" s="108"/>
@@ -4305,12 +4295,12 @@
         <v>9</v>
       </c>
       <c r="C30" s="111" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D30" s="106"/>
       <c r="E30" s="107"/>
-      <c r="F30" s="253" t="s">
-        <v>54</v>
+      <c r="F30" s="108" t="s">
+        <v>53</v>
       </c>
       <c r="G30" s="108"/>
       <c r="H30" s="108"/>
@@ -4322,14 +4312,14 @@
         <v>10</v>
       </c>
       <c r="C31" s="111" t="s">
-        <v>55</v>
-      </c>
-      <c r="D31" s="252" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" s="251" t="s">
         <v>26</v>
       </c>
       <c r="E31" s="107"/>
-      <c r="F31" s="253" t="s">
-        <v>54</v>
+      <c r="F31" s="108" t="s">
+        <v>53</v>
       </c>
       <c r="G31" s="108"/>
       <c r="H31" s="108"/>
@@ -4341,13 +4331,13 @@
         <v>11</v>
       </c>
       <c r="C32" s="113" t="s">
-        <v>56</v>
-      </c>
-      <c r="D32" s="252" t="s">
+        <v>55</v>
+      </c>
+      <c r="D32" s="251" t="s">
         <v>26</v>
       </c>
       <c r="E32" s="106"/>
-      <c r="F32" s="254" t="s">
+      <c r="F32" s="252" t="s">
         <v>35</v>
       </c>
       <c r="G32" s="114"/>
@@ -4360,13 +4350,13 @@
         <v>12</v>
       </c>
       <c r="C33" s="111" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D33" s="106"/>
-      <c r="E33" s="252" t="s">
+      <c r="E33" s="251" t="s">
         <v>26</v>
       </c>
-      <c r="F33" s="255" t="s">
+      <c r="F33" s="253" t="s">
         <v>35</v>
       </c>
       <c r="G33" s="117"/>
@@ -4379,9 +4369,9 @@
         <v>13</v>
       </c>
       <c r="C34" s="119" t="s">
-        <v>58</v>
-      </c>
-      <c r="D34" s="252" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" s="251" t="s">
         <v>26</v>
       </c>
       <c r="E34" s="106"/>
@@ -4396,9 +4386,9 @@
         <v>14</v>
       </c>
       <c r="C35" s="121" t="s">
-        <v>59</v>
-      </c>
-      <c r="D35" s="256" t="s">
+        <v>58</v>
+      </c>
+      <c r="D35" s="254" t="s">
         <v>26</v>
       </c>
       <c r="E35" s="122"/>
@@ -4411,7 +4401,7 @@
       <c r="A36" s="126"/>
       <c r="B36" s="127"/>
       <c r="C36" s="99" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D36" s="128"/>
       <c r="E36" s="128"/>
@@ -4422,13 +4412,13 @@
     </row>
     <row r="37" s="2" customFormat="1" ht="12" customHeight="1" spans="1:10">
       <c r="A37" s="38" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B37" s="93">
         <v>15</v>
       </c>
       <c r="C37" s="78" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D37" s="122" t="s">
         <v>26</v>
@@ -4443,7 +4433,7 @@
       <c r="A38" s="133"/>
       <c r="B38" s="93"/>
       <c r="C38" s="134" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D38" s="128"/>
       <c r="E38" s="128"/>
@@ -4456,10 +4446,10 @@
       <c r="A39" s="133"/>
       <c r="B39" s="98"/>
       <c r="C39" s="138" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D39" s="106"/>
-      <c r="E39" s="252" t="s">
+      <c r="E39" s="251" t="s">
         <v>26</v>
       </c>
       <c r="F39" s="139"/>
@@ -4469,16 +4459,16 @@
     </row>
     <row r="40" s="2" customFormat="1" ht="50.25" customHeight="1" spans="1:10">
       <c r="A40" s="38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B40" s="142">
         <v>16</v>
       </c>
       <c r="C40" s="143" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D40" s="79"/>
-      <c r="E40" s="252" t="s">
+      <c r="E40" s="251" t="s">
         <v>26</v>
       </c>
       <c r="F40" s="144"/>
@@ -4493,10 +4483,10 @@
         <v>17</v>
       </c>
       <c r="C41" s="111" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D41" s="107"/>
-      <c r="E41" s="252" t="s">
+      <c r="E41" s="251" t="s">
         <v>26</v>
       </c>
       <c r="F41" s="144"/>
@@ -4510,7 +4500,7 @@
         <v>18</v>
       </c>
       <c r="C42" s="78" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D42" s="149"/>
       <c r="E42" s="149"/>
@@ -4523,10 +4513,10 @@
       <c r="A43" s="133"/>
       <c r="B43" s="153"/>
       <c r="C43" s="138" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D43" s="79"/>
-      <c r="E43" s="252" t="s">
+      <c r="E43" s="251" t="s">
         <v>26</v>
       </c>
       <c r="F43" s="154"/>
@@ -4540,7 +4530,7 @@
         <v>19</v>
       </c>
       <c r="C44" s="113" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D44" s="149"/>
       <c r="E44" s="149"/>
@@ -4553,10 +4543,10 @@
       <c r="A45" s="133"/>
       <c r="B45" s="158"/>
       <c r="C45" s="134" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D45" s="106"/>
-      <c r="E45" s="252" t="s">
+      <c r="E45" s="251" t="s">
         <v>26</v>
       </c>
       <c r="F45" s="135"/>
@@ -4568,10 +4558,10 @@
       <c r="A46" s="133"/>
       <c r="B46" s="159"/>
       <c r="C46" s="160" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D46" s="106"/>
-      <c r="E46" s="252" t="s">
+      <c r="E46" s="251" t="s">
         <v>26</v>
       </c>
       <c r="F46" s="139"/>
@@ -4585,7 +4575,7 @@
         <v>20</v>
       </c>
       <c r="C47" s="161" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D47" s="88"/>
       <c r="E47" s="122" t="s">
@@ -4602,7 +4592,7 @@
       <c r="A48" s="133"/>
       <c r="B48" s="153"/>
       <c r="C48" s="138" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D48" s="100"/>
       <c r="E48" s="128"/>
@@ -4617,10 +4607,10 @@
         <v>21</v>
       </c>
       <c r="C49" s="162" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D49" s="106"/>
-      <c r="E49" s="252" t="s">
+      <c r="E49" s="251" t="s">
         <v>26</v>
       </c>
       <c r="F49" s="163" t="s">
@@ -4632,16 +4622,16 @@
     </row>
     <row r="50" s="2" customFormat="1" ht="35.25" customHeight="1" spans="1:9">
       <c r="A50" s="38" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B50" s="164">
         <v>22</v>
       </c>
       <c r="C50" s="111" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D50" s="106"/>
-      <c r="E50" s="252" t="s">
+      <c r="E50" s="251" t="s">
         <v>26</v>
       </c>
       <c r="F50" s="163" t="s">
@@ -4657,10 +4647,10 @@
         <v>23</v>
       </c>
       <c r="C51" s="165" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D51" s="106"/>
-      <c r="E51" s="252" t="s">
+      <c r="E51" s="251" t="s">
         <v>26</v>
       </c>
       <c r="F51" s="166" t="s">
@@ -4676,7 +4666,7 @@
         <v>24</v>
       </c>
       <c r="C52" s="113" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D52" s="149"/>
       <c r="E52" s="170"/>
@@ -4689,7 +4679,7 @@
       <c r="A53" s="133"/>
       <c r="B53" s="148"/>
       <c r="C53" s="174" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D53" s="106"/>
       <c r="E53" s="175"/>
@@ -4704,7 +4694,7 @@
       <c r="A54" s="133"/>
       <c r="B54" s="148"/>
       <c r="C54" s="174" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D54" s="106"/>
       <c r="E54" s="175"/>
@@ -4717,7 +4707,7 @@
       <c r="A55" s="133"/>
       <c r="B55" s="148"/>
       <c r="C55" s="174" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D55" s="106"/>
       <c r="E55" s="175"/>
@@ -4730,7 +4720,7 @@
       <c r="A56" s="133"/>
       <c r="B56" s="148"/>
       <c r="C56" s="174" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D56" s="106"/>
       <c r="E56" s="175"/>
@@ -4743,7 +4733,7 @@
       <c r="A57" s="133"/>
       <c r="B57" s="148"/>
       <c r="C57" s="174" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D57" s="106"/>
       <c r="E57" s="175"/>
@@ -4756,7 +4746,7 @@
       <c r="A58" s="133"/>
       <c r="B58" s="153"/>
       <c r="C58" s="162" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D58" s="106"/>
       <c r="E58" s="175"/>
@@ -4771,10 +4761,10 @@
         <v>25</v>
       </c>
       <c r="C59" s="174" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D59" s="88"/>
-      <c r="E59" s="257" t="s">
+      <c r="E59" s="255" t="s">
         <v>26</v>
       </c>
       <c r="F59" s="131" t="s">
@@ -4784,11 +4774,11 @@
       <c r="H59" s="131"/>
       <c r="I59" s="132"/>
     </row>
-    <row r="60" s="2" customFormat="1" ht="10.2" spans="1:9">
+    <row r="60" s="2" customFormat="1" ht="10.8" spans="1:9">
       <c r="A60" s="133"/>
       <c r="B60" s="179"/>
       <c r="C60" s="174" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D60" s="100"/>
       <c r="E60" s="100"/>
@@ -4797,14 +4787,14 @@
       <c r="H60" s="136"/>
       <c r="I60" s="137"/>
     </row>
-    <row r="61" s="2" customFormat="1" ht="30.6" spans="1:9">
+    <row r="61" s="2" customFormat="1" ht="21.6" spans="1:9">
       <c r="A61" s="133"/>
       <c r="B61" s="179"/>
       <c r="C61" s="134" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D61" s="180"/>
-      <c r="E61" s="250" t="s">
+      <c r="E61" s="249" t="s">
         <v>26</v>
       </c>
       <c r="F61" s="136"/>
@@ -4812,14 +4802,14 @@
       <c r="H61" s="136"/>
       <c r="I61" s="137"/>
     </row>
-    <row r="62" s="2" customFormat="1" ht="30.6" spans="1:9">
+    <row r="62" s="2" customFormat="1" ht="21.6" spans="1:9">
       <c r="A62" s="133"/>
       <c r="B62" s="181"/>
       <c r="C62" s="134" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D62" s="180"/>
-      <c r="E62" s="250" t="s">
+      <c r="E62" s="249" t="s">
         <v>26</v>
       </c>
       <c r="F62" s="136"/>
@@ -4833,10 +4823,10 @@
         <v>26</v>
       </c>
       <c r="C63" s="113" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D63" s="88"/>
-      <c r="E63" s="257" t="s">
+      <c r="E63" s="255" t="s">
         <v>26</v>
       </c>
       <c r="F63" s="182"/>
@@ -4848,7 +4838,7 @@
       <c r="A64" s="133"/>
       <c r="B64" s="148"/>
       <c r="C64" s="138" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D64" s="100"/>
       <c r="E64" s="100"/>
@@ -4863,10 +4853,10 @@
         <v>27</v>
       </c>
       <c r="C65" s="185" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D65" s="79"/>
-      <c r="E65" s="250" t="s">
+      <c r="E65" s="249" t="s">
         <v>26</v>
       </c>
       <c r="F65" s="182"/>
@@ -4874,17 +4864,17 @@
       <c r="H65" s="183"/>
       <c r="I65" s="184"/>
     </row>
-    <row r="66" s="2" customFormat="1" ht="40.8" spans="1:9">
+    <row r="66" s="2" customFormat="1" ht="32.4" spans="1:9">
       <c r="A66" s="38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B66" s="186">
         <v>28</v>
       </c>
       <c r="C66" s="162" t="s">
-        <v>94</v>
-      </c>
-      <c r="D66" s="258" t="s">
+        <v>93</v>
+      </c>
+      <c r="D66" s="256" t="s">
         <v>26</v>
       </c>
       <c r="E66" s="188"/>
@@ -4899,9 +4889,9 @@
         <v>29</v>
       </c>
       <c r="C67" s="193" t="s">
-        <v>95</v>
-      </c>
-      <c r="D67" s="258" t="s">
+        <v>94</v>
+      </c>
+      <c r="D67" s="256" t="s">
         <v>26</v>
       </c>
       <c r="E67" s="187"/>
@@ -4916,9 +4906,9 @@
         <v>30</v>
       </c>
       <c r="C68" s="193" t="s">
-        <v>96</v>
-      </c>
-      <c r="D68" s="258" t="s">
+        <v>95</v>
+      </c>
+      <c r="D68" s="256" t="s">
         <v>26</v>
       </c>
       <c r="E68" s="187"/>
@@ -4933,9 +4923,9 @@
         <v>31</v>
       </c>
       <c r="C69" s="111" t="s">
-        <v>97</v>
-      </c>
-      <c r="D69" s="258" t="s">
+        <v>96</v>
+      </c>
+      <c r="D69" s="256" t="s">
         <v>26</v>
       </c>
       <c r="E69" s="187"/>
@@ -4950,9 +4940,9 @@
         <v>32</v>
       </c>
       <c r="C70" s="111" t="s">
-        <v>98</v>
-      </c>
-      <c r="D70" s="258" t="s">
+        <v>97</v>
+      </c>
+      <c r="D70" s="256" t="s">
         <v>26</v>
       </c>
       <c r="E70" s="107"/>
@@ -4967,7 +4957,7 @@
         <v>33</v>
       </c>
       <c r="C71" s="193" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D71" s="107"/>
       <c r="E71" s="107"/>
@@ -4978,13 +4968,13 @@
       <c r="H71" s="144"/>
       <c r="I71" s="145"/>
     </row>
-    <row r="72" s="2" customFormat="1" ht="61.2" spans="1:9">
+    <row r="72" s="2" customFormat="1" ht="54" spans="1:9">
       <c r="A72" s="133"/>
       <c r="B72" s="194">
         <v>34</v>
       </c>
       <c r="C72" s="195" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D72" s="107"/>
       <c r="E72" s="107"/>
@@ -4999,7 +4989,7 @@
         <v>35</v>
       </c>
       <c r="C73" s="197" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D73" s="198"/>
       <c r="E73" s="198"/>
@@ -5008,9 +4998,9 @@
       <c r="H73" s="200"/>
       <c r="I73" s="201"/>
     </row>
-    <row r="74" s="2" customFormat="1" ht="10.95" spans="1:9">
+    <row r="74" s="2" customFormat="1" ht="11.55" spans="1:9">
       <c r="A74" s="202" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B74" s="203"/>
       <c r="C74" s="204"/>
@@ -5034,21 +5024,21 @@
     </row>
     <row r="76" s="2" customFormat="1" ht="11.4" spans="1:9">
       <c r="A76" s="211" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B76" s="212"/>
       <c r="I76" s="213"/>
     </row>
     <row r="77" s="2" customFormat="1" ht="15.75" customHeight="1" spans="1:9">
       <c r="A77" s="214" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B77" s="203"/>
       <c r="I77" s="213"/>
     </row>
-    <row r="78" s="2" customFormat="1" ht="10.2" spans="1:9">
+    <row r="78" s="2" customFormat="1" ht="10.8" spans="1:9">
       <c r="A78" s="214" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B78" s="203"/>
       <c r="C78" s="215"/>
@@ -5061,7 +5051,7 @@
     </row>
     <row r="79" s="2" customFormat="1" ht="13.5" customHeight="1" spans="1:9">
       <c r="A79" s="216" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B79" s="217"/>
       <c r="F79" s="218"/>
@@ -5091,16 +5081,16 @@
       <c r="H81" s="222"/>
       <c r="I81" s="223"/>
     </row>
-    <row r="82" s="2" customFormat="1" ht="10.2" spans="1:10">
+    <row r="82" s="2" customFormat="1" ht="10.8" spans="1:10">
       <c r="A82" s="224" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B82" s="207"/>
       <c r="C82" s="224" t="s">
+        <v>107</v>
+      </c>
+      <c r="D82" s="224" t="s">
         <v>108</v>
-      </c>
-      <c r="D82" s="224" t="s">
-        <v>109</v>
       </c>
       <c r="E82" s="208"/>
       <c r="F82" s="208"/>
@@ -5121,15 +5111,15 @@
     </row>
     <row r="84" s="2" customFormat="1" ht="15" customHeight="1" spans="1:10">
       <c r="A84" s="228" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B84" s="229"/>
       <c r="C84" s="228" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D84" s="216"/>
       <c r="E84" s="230" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F84" s="230"/>
       <c r="G84" s="230"/>
@@ -5139,14 +5129,14 @@
     </row>
     <row r="85" s="3" customFormat="1" ht="14.25" customHeight="1" spans="1:10">
       <c r="A85" s="233" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B85" s="234"/>
       <c r="C85" s="233" t="s">
+        <v>113</v>
+      </c>
+      <c r="D85" s="233" t="s">
         <v>114</v>
-      </c>
-      <c r="D85" s="233" t="s">
-        <v>115</v>
       </c>
       <c r="E85" s="235"/>
       <c r="F85" s="235"/>
@@ -5156,14 +5146,14 @@
     </row>
     <row r="86" s="3" customFormat="1" ht="14.25" customHeight="1" spans="1:10">
       <c r="A86" s="236" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B86" s="237"/>
       <c r="C86" s="238" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D86" s="239" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E86" s="240"/>
       <c r="F86" s="240"/>
@@ -5173,7 +5163,7 @@
     </row>
     <row r="87" s="2" customFormat="1" ht="12.75" customHeight="1" spans="1:10">
       <c r="A87" s="242" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B87" s="243"/>
     </row>

</xml_diff>